<commit_message>
added the option to choose between PPP or EXCH to predict_impacts.py and func_data_upload_OECD_salaries.py
</commit_message>
<xml_diff>
--- a/OECD_salaries/impact_multipliers.xlsx
+++ b/OECD_salaries/impact_multipliers.xlsx
@@ -1068,139 +1068,139 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5323020388218841</v>
+        <v>0.532299461192109</v>
       </c>
       <c r="C5" t="n">
-        <v>0.49664399438928</v>
+        <v>0.4966411979375981</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6488589359082929</v>
+        <v>0.648859462226913</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6038044842023343</v>
+        <v>0.6038040197822913</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9822639317050121</v>
+        <v>0.9822668347553692</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7120863165196017</v>
+        <v>0.7120856637249304</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8638795157747572</v>
+        <v>0.8638961726672973</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8320989531145501</v>
+        <v>0.8321018591804967</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8091667393674794</v>
+        <v>0.8091677673163344</v>
       </c>
       <c r="K5" t="n">
-        <v>0.3961651808929453</v>
+        <v>0.3961645993181257</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5563228184335853</v>
+        <v>0.5563205317042155</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7516917435215303</v>
+        <v>0.7517042079404832</v>
       </c>
       <c r="N5" t="n">
-        <v>0.7710350647395643</v>
+        <v>0.7710320930967193</v>
       </c>
       <c r="O5" t="n">
-        <v>0.8105003934089549</v>
+        <v>0.8105013609413128</v>
       </c>
       <c r="P5" t="n">
-        <v>0.5011077835870424</v>
+        <v>0.5011058146745573</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.8854289900026628</v>
+        <v>0.8854258868538426</v>
       </c>
       <c r="R5" t="n">
-        <v>0.7963186354670579</v>
+        <v>0.7963144424117916</v>
       </c>
       <c r="S5" t="n">
-        <v>0.7329510242650783</v>
+        <v>0.7329647462302041</v>
       </c>
       <c r="T5" t="n">
-        <v>0.8439562095473179</v>
+        <v>0.8439611630112283</v>
       </c>
       <c r="U5" t="n">
-        <v>0.4962174284914603</v>
+        <v>0.496215288750485</v>
       </c>
       <c r="V5" t="n">
-        <v>0.7212972793193562</v>
+        <v>0.7212998611353432</v>
       </c>
       <c r="W5" t="n">
-        <v>0.6845614129611656</v>
+        <v>0.6845618487748063</v>
       </c>
       <c r="X5" t="n">
-        <v>0.6271853832609694</v>
+        <v>0.6271848671552691</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.6326802467519861</v>
+        <v>0.6326872072524156</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.8887242421952316</v>
+        <v>0.8887240175339782</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.070720931847378</v>
+        <v>1.07072094109013</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.8246007040582655</v>
+        <v>0.8246021682247652</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.7389485061779489</v>
+        <v>0.7389262997137055</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.7608022797340757</v>
+        <v>0.7608027149380651</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.8581353108992953</v>
+        <v>0.8581402944054395</v>
       </c>
       <c r="AF5" t="n">
-        <v>1.081325603395995</v>
+        <v>1.081321765263725</v>
       </c>
       <c r="AG5" t="n">
-        <v>1.023426452577572</v>
+        <v>1.023426249356288</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.9573770610958279</v>
+        <v>0.9573745007430758</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.2335069379051387</v>
+        <v>0.2335067779243715</v>
       </c>
       <c r="AJ5" t="n">
-        <v>1.064386342184649</v>
+        <v>1.064385847237328</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.9597118647355001</v>
+        <v>0.9597116340953997</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.2664727484253964</v>
+        <v>0.2664728191391146</v>
       </c>
       <c r="AM5" t="n">
-        <v>1.000199455183104</v>
+        <v>1.000199402799596</v>
       </c>
       <c r="AN5" t="n">
-        <v>1.002529064462174</v>
+        <v>1.002528280665804</v>
       </c>
       <c r="AO5" t="n">
-        <v>1.214866875875565</v>
+        <v>1.214867257437397</v>
       </c>
       <c r="AP5" t="n">
-        <v>1.306923707320978</v>
+        <v>1.306923726314887</v>
       </c>
       <c r="AQ5" t="n">
-        <v>1.129606393725642</v>
+        <v>1.129607212529946</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.9184905664330304</v>
+        <v>0.9184907699582012</v>
       </c>
       <c r="AS5" t="n">
-        <v>1.08037128564953</v>
+        <v>1.080368936487522</v>
       </c>
       <c r="AT5" t="n">
-        <v>1.876296961851884</v>
+        <v>1.876329838646918</v>
       </c>
     </row>
     <row r="6">
@@ -1210,139 +1210,139 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.311660754039187</v>
+        <v>2.311658176409411</v>
       </c>
       <c r="C6" t="n">
-        <v>2.07903000292915</v>
+        <v>2.079027206477469</v>
       </c>
       <c r="D6" t="n">
-        <v>2.300992681258934</v>
+        <v>2.300993207577555</v>
       </c>
       <c r="E6" t="n">
-        <v>2.070094159910667</v>
+        <v>2.070093695490623</v>
       </c>
       <c r="F6" t="n">
-        <v>2.443683341688319</v>
+        <v>2.443686244738676</v>
       </c>
       <c r="G6" t="n">
-        <v>2.731532501866206</v>
+        <v>2.731531849071537</v>
       </c>
       <c r="H6" t="n">
-        <v>2.481278951802902</v>
+        <v>2.481295608695443</v>
       </c>
       <c r="I6" t="n">
-        <v>2.903587898463966</v>
+        <v>2.903590804529913</v>
       </c>
       <c r="J6" t="n">
-        <v>2.627040392658938</v>
+        <v>2.627041420607794</v>
       </c>
       <c r="K6" t="n">
-        <v>2.244163377549451</v>
+        <v>2.244162795974631</v>
       </c>
       <c r="L6" t="n">
-        <v>2.274873613585684</v>
+        <v>2.274871326856314</v>
       </c>
       <c r="M6" t="n">
-        <v>2.388117772933273</v>
+        <v>2.388130237352225</v>
       </c>
       <c r="N6" t="n">
-        <v>2.450179928834807</v>
+        <v>2.450176957191962</v>
       </c>
       <c r="O6" t="n">
-        <v>2.64560362522562</v>
+        <v>2.64560459275798</v>
       </c>
       <c r="P6" t="n">
-        <v>2.300120089217605</v>
+        <v>2.30011812030512</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.515149840337779</v>
+        <v>2.515146737188959</v>
       </c>
       <c r="R6" t="n">
-        <v>2.235750376703802</v>
+        <v>2.235746183648536</v>
       </c>
       <c r="S6" t="n">
-        <v>2.306759131203252</v>
+        <v>2.306772853168378</v>
       </c>
       <c r="T6" t="n">
-        <v>2.412715175499637</v>
+        <v>2.412720128963548</v>
       </c>
       <c r="U6" t="n">
-        <v>2.100612625434847</v>
+        <v>2.10061048569387</v>
       </c>
       <c r="V6" t="n">
-        <v>2.255429867136213</v>
+        <v>2.255432448952201</v>
       </c>
       <c r="W6" t="n">
-        <v>2.312822299797904</v>
+        <v>2.312822735611544</v>
       </c>
       <c r="X6" t="n">
-        <v>1.970535080813035</v>
+        <v>1.970534564707335</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.203727325786012</v>
+        <v>2.203734286286442</v>
       </c>
       <c r="Z6" t="n">
-        <v>2.541178271520445</v>
+        <v>2.541178046859192</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.602193912160325</v>
+        <v>2.602193921403078</v>
       </c>
       <c r="AB6" t="n">
-        <v>2.515368558915256</v>
+        <v>2.515370023081756</v>
       </c>
       <c r="AC6" t="n">
-        <v>2.48597955838162</v>
+        <v>2.485957351917377</v>
       </c>
       <c r="AD6" t="n">
-        <v>2.531061588827494</v>
+        <v>2.531062024031483</v>
       </c>
       <c r="AE6" t="n">
-        <v>2.497167745368922</v>
+        <v>2.497172728875066</v>
       </c>
       <c r="AF6" t="n">
-        <v>2.669105004190663</v>
+        <v>2.669101166058393</v>
       </c>
       <c r="AG6" t="n">
-        <v>2.738746164596603</v>
+        <v>2.738745961375319</v>
       </c>
       <c r="AH6" t="n">
-        <v>2.62688620671033</v>
+        <v>2.626883646357579</v>
       </c>
       <c r="AI6" t="n">
-        <v>1.719139253515531</v>
+        <v>1.719139093534764</v>
       </c>
       <c r="AJ6" t="n">
-        <v>2.597414619743147</v>
+        <v>2.597414124795826</v>
       </c>
       <c r="AK6" t="n">
-        <v>2.584393565187041</v>
+        <v>2.584393334546941</v>
       </c>
       <c r="AL6" t="n">
-        <v>1.612833317986191</v>
+        <v>1.61283338869991</v>
       </c>
       <c r="AM6" t="n">
-        <v>2.47522260601862</v>
+        <v>2.475222553635112</v>
       </c>
       <c r="AN6" t="n">
-        <v>2.486069041241215</v>
+        <v>2.486068257444845</v>
       </c>
       <c r="AO6" t="n">
-        <v>2.80075265312137</v>
+        <v>2.800753034683203</v>
       </c>
       <c r="AP6" t="n">
-        <v>2.578454712169853</v>
+        <v>2.578454731163763</v>
       </c>
       <c r="AQ6" t="n">
-        <v>2.51701097106052</v>
+        <v>2.517011789864824</v>
       </c>
       <c r="AR6" t="n">
-        <v>2.542763281551146</v>
+        <v>2.542763485076317</v>
       </c>
       <c r="AS6" t="n">
-        <v>2.664237482764956</v>
+        <v>2.664235133602948</v>
       </c>
       <c r="AT6" t="n">
-        <v>2.876296961851884</v>
+        <v>2.876329838646918</v>
       </c>
     </row>
     <row r="8">
@@ -1591,139 +1591,139 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1072154877798823</v>
+        <v>0.1046367107946674</v>
       </c>
       <c r="C10" t="n">
-        <v>0.1244590669275001</v>
+        <v>0.1214654099235284</v>
       </c>
       <c r="D10" t="n">
-        <v>0.151945649966621</v>
+        <v>0.1482928063056545</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1936672243133974</v>
+        <v>0.1890108741112505</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4015822800879496</v>
+        <v>0.3919291528504908</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1500936785977638</v>
+        <v>0.1464851494710483</v>
       </c>
       <c r="H10" t="n">
-        <v>0.287618791120003</v>
+        <v>0.2807125543457351</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2222148841837386</v>
+        <v>0.216874259775368</v>
       </c>
       <c r="J10" t="n">
-        <v>0.230031066620642</v>
+        <v>0.2245012081463583</v>
       </c>
       <c r="K10" t="n">
-        <v>0.02560409448105623</v>
+        <v>0.02498811060534004</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1233468124577887</v>
+        <v>0.120380265193937</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2255082101087876</v>
+        <v>0.2200931353963115</v>
       </c>
       <c r="N10" t="n">
-        <v>0.2430756868149671</v>
+        <v>0.2372303611313924</v>
       </c>
       <c r="O10" t="n">
-        <v>0.2165242165242165</v>
+        <v>0.2113190762979792</v>
       </c>
       <c r="P10" t="n">
-        <v>0.09781387441327569</v>
+        <v>0.09546143327050302</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3246069691500062</v>
+        <v>0.3168014660291828</v>
       </c>
       <c r="R10" t="n">
-        <v>0.297668026477163</v>
+        <v>0.2905094505379804</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2489514535023863</v>
+        <v>0.2429735332401292</v>
       </c>
       <c r="T10" t="n">
-        <v>0.3033897591080468</v>
+        <v>0.2960984069255559</v>
       </c>
       <c r="U10" t="n">
-        <v>0.1180239098765624</v>
+        <v>0.1151855192829111</v>
       </c>
       <c r="V10" t="n">
-        <v>0.2447495122295006</v>
+        <v>0.2388665919864685</v>
       </c>
       <c r="W10" t="n">
-        <v>0.2048975988700565</v>
+        <v>0.1999717514124294</v>
       </c>
       <c r="X10" t="n">
-        <v>0.2428087277534926</v>
+        <v>0.2369709835248989</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.1716548155261373</v>
+        <v>0.1675316856056276</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.293361163815513</v>
+        <v>0.2863081317829606</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.4269109538148684</v>
+        <v>0.4166473739783348</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.2644575559108457</v>
+        <v>0.2581002080340646</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.2015067132927514</v>
+        <v>0.1966498294694124</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.2142098131708113</v>
+        <v>0.2090597819670196</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.2886842896768372</v>
+        <v>0.2817464826387729</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.4255738832236991</v>
+        <v>0.4153403487183199</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.3706674783641734</v>
+        <v>0.3617560445113635</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.3164763947354399</v>
+        <v>0.3088666275909842</v>
       </c>
       <c r="AI10" t="n">
         <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.4088317554705986</v>
+        <v>0.3990026594221656</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.3242297512529251</v>
+        <v>0.3164347318808828</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.04193350222231011</v>
+        <v>0.04092541300490976</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.3976766829531524</v>
+        <v>0.3881159488295433</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.3991258597044782</v>
+        <v>0.3895299079201081</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.4648480573954492</v>
+        <v>0.4536725011746079</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.634801193636698</v>
+        <v>0.6195396395232946</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.495548530924531</v>
+        <v>0.4836352152882653</v>
       </c>
       <c r="AR10" t="n">
-        <v>0.3178654499113278</v>
+        <v>0.3102235966170875</v>
       </c>
       <c r="AS10" t="n">
-        <v>0.4262312810921537</v>
+        <v>0.4159827983256358</v>
       </c>
       <c r="AT10" t="n">
-        <v>1.024615744714052</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1733,136 +1733,136 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.183466137255626</v>
+        <v>0.1790551275102479</v>
       </c>
       <c r="C11" t="n">
-        <v>0.146750270674734</v>
+        <v>0.1432221666998557</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2023858313218538</v>
+        <v>0.197520306539594</v>
       </c>
       <c r="E11" t="n">
-        <v>0.136060741899392</v>
+        <v>0.1327897002577596</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1348163339653053</v>
+        <v>0.1315751983161005</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2387652634224246</v>
+        <v>0.2330247048509609</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1841319878852239</v>
+        <v>0.179705520810113</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2321810381332488</v>
+        <v>0.2265988663465042</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2118419407505115</v>
+        <v>0.2067490713353405</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1907353710211243</v>
+        <v>0.1861499266194013</v>
       </c>
       <c r="L11" t="n">
-        <v>0.18045217592204</v>
+        <v>0.1761137308219215</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1849786217962978</v>
+        <v>0.1805316334783131</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1779742232584578</v>
+        <v>0.1736953072749344</v>
       </c>
       <c r="O11" t="n">
-        <v>0.226077077976683</v>
+        <v>0.2206419490224901</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1758330670363787</v>
+        <v>0.1716055846669838</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.1589116328774511</v>
+        <v>0.1550909851894961</v>
       </c>
       <c r="R11" t="n">
-        <v>0.137188836960623</v>
+        <v>0.1338905808477802</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1513013715222133</v>
+        <v>0.1476639395182687</v>
       </c>
       <c r="T11" t="n">
-        <v>0.1574812211966344</v>
+        <v>0.1536951984566596</v>
       </c>
       <c r="U11" t="n">
-        <v>0.1529524869151545</v>
+        <v>0.1492750667664597</v>
       </c>
       <c r="V11" t="n">
-        <v>0.14913938917371</v>
+        <v>0.1455540180143268</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1689304337945714</v>
+        <v>0.1648691388590092</v>
       </c>
       <c r="X11" t="n">
-        <v>0.09968717327351939</v>
+        <v>0.09729053821669019</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.1738417425196833</v>
+        <v>0.169662337652387</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.1919569227007842</v>
+        <v>0.1873420757812198</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.1577926124494617</v>
+        <v>0.1539990651691983</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.1858436925900771</v>
+        <v>0.1813759177730122</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.2020212406274891</v>
+        <v>0.1971648850301281</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.2012521367651361</v>
+        <v>0.1964140847635253</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.1799296709697155</v>
+        <v>0.1756039664828334</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.1649207244680556</v>
+        <v>0.1609558562407721</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.1882093296187449</v>
+        <v>0.1836844363021344</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.2063318975397187</v>
+        <v>0.2013712213329924</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.1275144020067215</v>
+        <v>0.12444868333638</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.1724125927505868</v>
+        <v>0.1682674576511157</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.1998535399262782</v>
+        <v>0.1950487047346534</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.1035830013616472</v>
+        <v>0.1010926979106405</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.1485162334514762</v>
+        <v>0.1449456601681967</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.1483392190469949</v>
+        <v>0.1447728889638126</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.1985713021525722</v>
+        <v>0.1937974864654529</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.07888892838932765</v>
+        <v>0.07699233443782527</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.1213114437345973</v>
+        <v>0.1183949764527252</v>
       </c>
       <c r="AR11" t="n">
-        <v>0.1837075499243461</v>
+        <v>0.1792909604932735</v>
       </c>
       <c r="AS11" t="n">
-        <v>0.1637421889500873</v>
+        <v>0.159805591452683</v>
       </c>
       <c r="AT11" t="n">
         <v>0</v>
@@ -1875,139 +1875,139 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1342275933983704</v>
+        <v>0.1309999509322364</v>
       </c>
       <c r="C12" t="n">
-        <v>0.125235906084766</v>
+        <v>0.1222243817700805</v>
       </c>
       <c r="D12" t="n">
-        <v>0.163619086665082</v>
+        <v>0.1596855978837181</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1522579604936349</v>
+        <v>0.1485973643238769</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2476919380707144</v>
+        <v>0.2417378121464536</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1795627774973062</v>
+        <v>0.1752456912103629</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2178396097171366</v>
+        <v>0.2126065579260827</v>
       </c>
       <c r="I12" t="n">
-        <v>0.20982568504353</v>
+        <v>0.2047819144493315</v>
       </c>
       <c r="J12" t="n">
-        <v>0.2040429984519495</v>
+        <v>0.1991377890501582</v>
       </c>
       <c r="K12" t="n">
-        <v>0.09989873218818095</v>
+        <v>0.09749689198545619</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1402847774849979</v>
+        <v>0.1369115839280287</v>
       </c>
       <c r="M12" t="n">
-        <v>0.189549853939376</v>
+        <v>0.1849958933552621</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1944275498076369</v>
+        <v>0.1897525241461716</v>
       </c>
       <c r="O12" t="n">
-        <v>0.2043792984458579</v>
+        <v>0.1994659890807284</v>
       </c>
       <c r="P12" t="n">
-        <v>0.1263615145509282</v>
+        <v>0.1233231327854639</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2232736187076221</v>
+        <v>0.217905063199235</v>
       </c>
       <c r="R12" t="n">
-        <v>0.2008031647851413</v>
+        <v>0.1959745603517103</v>
       </c>
       <c r="S12" t="n">
-        <v>0.1848241127982833</v>
+        <v>0.180384074739017</v>
       </c>
       <c r="T12" t="n">
-        <v>0.2128156623105724</v>
+        <v>0.2077005125941371</v>
       </c>
       <c r="U12" t="n">
-        <v>0.1251283413757955</v>
+        <v>0.1221195646761678</v>
       </c>
       <c r="V12" t="n">
-        <v>0.181885453871474</v>
+        <v>0.1775133234299047</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1726219783011428</v>
+        <v>0.1684720258757046</v>
       </c>
       <c r="X12" t="n">
-        <v>0.1581537895215995</v>
+        <v>0.1543514371379933</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.1595393981585383</v>
+        <v>0.155705573926192</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.2241045638086933</v>
+        <v>0.2187167396873124</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.2699976393124901</v>
+        <v>0.2635065427847635</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.2079348940036267</v>
+        <v>0.2029362256616564</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.1863364638788777</v>
+        <v>0.1818512248504777</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.1918472063092545</v>
+        <v>0.1872350539352307</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.21639112607404</v>
+        <v>0.2111900248937429</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.2726717593363425</v>
+        <v>0.2661154265951511</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.2580716580642022</v>
+        <v>0.2518672255428988</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.2414163567175396</v>
+        <v>0.2356117594788512</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.05888212336401988</v>
+        <v>0.05746648020633152</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.2684002816779483</v>
+        <v>0.2619474636491025</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.2420051109411843</v>
+        <v>0.2361869326225377</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.06719492528443777</v>
+        <v>0.06557948819602565</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.2522146375481248</v>
+        <v>0.2461510526344706</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.2528020819392456</v>
+        <v>0.2467241940866849</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.3063461064494232</v>
+        <v>0.2989812365337762</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.3295595567832699</v>
+        <v>0.3216365157236864</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.2848464530641046</v>
+        <v>0.2779985707344482</v>
       </c>
       <c r="AR12" t="n">
-        <v>0.2316105693757549</v>
+        <v>0.2260423963735924</v>
       </c>
       <c r="AS12" t="n">
-        <v>0.272431114429686</v>
+        <v>0.2658809335474784</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.4731351889003855</v>
+        <v>0.4617684869433437</v>
       </c>
     </row>
     <row r="13">
@@ -2017,139 +2017,139 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4249092184338788</v>
+        <v>0.4146917892371519</v>
       </c>
       <c r="C13" t="n">
-        <v>0.3964452436869998</v>
+        <v>0.3869119583934644</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5179505679535568</v>
+        <v>0.5054987107289665</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4819859267064244</v>
+        <v>0.4703979386928872</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7840905521239692</v>
+        <v>0.7652421633130447</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5684217195174948</v>
+        <v>0.5547555455323721</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6895903887223636</v>
+        <v>0.6730246330819309</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6642216073605175</v>
+        <v>0.6482550405712039</v>
       </c>
       <c r="J13" t="n">
-        <v>0.6459160058231028</v>
+        <v>0.630388068531857</v>
       </c>
       <c r="K13" t="n">
-        <v>0.3162381976903615</v>
+        <v>0.3086349292101975</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4440837658648268</v>
+        <v>0.433405579943887</v>
       </c>
       <c r="M13" t="n">
-        <v>0.6000366858444615</v>
+        <v>0.5856206622298866</v>
       </c>
       <c r="N13" t="n">
-        <v>0.6154774598810618</v>
+        <v>0.6006781925524984</v>
       </c>
       <c r="O13" t="n">
-        <v>0.6469805929467575</v>
+        <v>0.6314270144011979</v>
       </c>
       <c r="P13" t="n">
-        <v>0.4000084560005823</v>
+        <v>0.3903901507229506</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.7067922207350794</v>
+        <v>0.6897975144179138</v>
       </c>
       <c r="R13" t="n">
-        <v>0.6356600282229271</v>
+        <v>0.6203745917374709</v>
       </c>
       <c r="S13" t="n">
-        <v>0.5850769378228828</v>
+        <v>0.5710215474974147</v>
       </c>
       <c r="T13" t="n">
-        <v>0.6736866426152537</v>
+        <v>0.6574941179763525</v>
       </c>
       <c r="U13" t="n">
-        <v>0.3961047381675123</v>
+        <v>0.3865801507255385</v>
       </c>
       <c r="V13" t="n">
-        <v>0.5757743552746846</v>
+        <v>0.5619339334307002</v>
       </c>
       <c r="W13" t="n">
-        <v>0.5464500109657707</v>
+        <v>0.533312916147143</v>
       </c>
       <c r="X13" t="n">
-        <v>0.5006496905486115</v>
+        <v>0.4886129588795822</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.505035956204359</v>
+        <v>0.4928995971842066</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.7094226503249902</v>
+        <v>0.6923669472514928</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.8547012055768205</v>
+        <v>0.8341529819322964</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.6582361425045496</v>
+        <v>0.6424123514687331</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.5898644177991181</v>
+        <v>0.5756659393500182</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.6073091562452018</v>
+        <v>0.5927089206657754</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.6850050867205926</v>
+        <v>0.668540474015349</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.8631663670280973</v>
+        <v>0.842411631554243</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.8169484660471207</v>
+        <v>0.7973077063563967</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.7642246489926983</v>
+        <v>0.7458496084028278</v>
       </c>
       <c r="AI13" t="n">
-        <v>0.1863965253707414</v>
+        <v>0.1819151635427116</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.8496446298991337</v>
+        <v>0.8292175807223838</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.7660884021203876</v>
+        <v>0.747670369238074</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.2127114288683951</v>
+        <v>0.2075975991115759</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.7984075539527534</v>
+        <v>0.7792126616322106</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.8002671606907188</v>
+        <v>0.7810269909706055</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.9697654659974446</v>
+        <v>0.946451224173837</v>
       </c>
       <c r="AP13" t="n">
-        <v>1.043249678809295</v>
+        <v>1.018168489684806</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.9017064277232331</v>
+        <v>0.8800287624754387</v>
       </c>
       <c r="AR13" t="n">
-        <v>0.7331835692114287</v>
+        <v>0.7155569534839534</v>
       </c>
       <c r="AS13" t="n">
-        <v>0.862404584471927</v>
+        <v>0.8416693233257972</v>
       </c>
       <c r="AT13" t="n">
-        <v>1.497750933614437</v>
+        <v>1.461768486943344</v>
       </c>
     </row>
     <row r="15">
@@ -2682,139 +2682,139 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.2969922616070581</v>
+        <v>0.2969908234459378</v>
       </c>
       <c r="C19" t="n">
-        <v>0.277097234933926</v>
+        <v>0.2770956746834498</v>
       </c>
       <c r="D19" t="n">
-        <v>0.362023942771024</v>
+        <v>0.3620242364249007</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3368862905891278</v>
+        <v>0.336886031470904</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5480437144628857</v>
+        <v>0.5480453341889587</v>
       </c>
       <c r="G19" t="n">
-        <v>0.3973009873692435</v>
+        <v>0.3973006231493992</v>
       </c>
       <c r="H19" t="n">
-        <v>0.4819923885953891</v>
+        <v>0.4820016821314382</v>
       </c>
       <c r="I19" t="n">
-        <v>0.4642607616407195</v>
+        <v>0.4642623830493088</v>
       </c>
       <c r="J19" t="n">
-        <v>0.4514659768612495</v>
+        <v>0.4514665503943812</v>
       </c>
       <c r="K19" t="n">
-        <v>0.2210361495209961</v>
+        <v>0.2210358250375107</v>
       </c>
       <c r="L19" t="n">
-        <v>0.3103944001339611</v>
+        <v>0.3103931242776283</v>
       </c>
       <c r="M19" t="n">
-        <v>0.4193984141670994</v>
+        <v>0.4194053685570969</v>
       </c>
       <c r="N19" t="n">
-        <v>0.4301908145273358</v>
+        <v>0.4301891565308132</v>
       </c>
       <c r="O19" t="n">
-        <v>0.452210074950477</v>
+        <v>0.4522106147748666</v>
       </c>
       <c r="P19" t="n">
-        <v>0.2795877586450787</v>
+        <v>0.2795866601112963</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.4940156885653713</v>
+        <v>0.4940139571964887</v>
       </c>
       <c r="R19" t="n">
-        <v>0.4442975139276981</v>
+        <v>0.4442951744571044</v>
       </c>
       <c r="S19" t="n">
-        <v>0.4089422291627449</v>
+        <v>0.4089498851872561</v>
       </c>
       <c r="T19" t="n">
-        <v>0.4708763917672101</v>
+        <v>0.4708791554997194</v>
       </c>
       <c r="U19" t="n">
-        <v>0.2768592370277027</v>
+        <v>0.2768580431819815</v>
       </c>
       <c r="V19" t="n">
-        <v>0.4024401461061368</v>
+        <v>0.4024415866029094</v>
       </c>
       <c r="W19" t="n">
-        <v>0.3819437601521007</v>
+        <v>0.3819440033096866</v>
       </c>
       <c r="X19" t="n">
-        <v>0.3499314145664829</v>
+        <v>0.3499311266107963</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.3529972152142336</v>
+        <v>0.3530010987514244</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.4958542394816943</v>
+        <v>0.4958541141343373</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.5973973569651788</v>
+        <v>0.5973973621220742</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.4600771933225371</v>
+        <v>0.4600780102386645</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.4122884604136962</v>
+        <v>0.412276070553134</v>
       </c>
       <c r="AD19" t="n">
-        <v>0.4244815409576811</v>
+        <v>0.4244817837751189</v>
       </c>
       <c r="AE19" t="n">
-        <v>0.4787874705738959</v>
+        <v>0.4787902510681502</v>
       </c>
       <c r="AF19" t="n">
-        <v>0.6033141206766131</v>
+        <v>0.603311979231531</v>
       </c>
       <c r="AG19" t="n">
-        <v>0.5710099052263966</v>
+        <v>0.5710097918412425</v>
       </c>
       <c r="AH19" t="n">
-        <v>0.5341583496746865</v>
+        <v>0.5341569211530974</v>
       </c>
       <c r="AI19" t="n">
-        <v>0.1302827126923545</v>
+        <v>0.1302826234327868</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.5938630400302851</v>
+        <v>0.5938627638796911</v>
       </c>
       <c r="AK19" t="n">
-        <v>0.5354610285351499</v>
+        <v>0.5354608998519587</v>
       </c>
       <c r="AL19" t="n">
-        <v>0.1486756360856032</v>
+        <v>0.1486756755395703</v>
       </c>
       <c r="AM19" t="n">
-        <v>0.558050649045842</v>
+        <v>0.5580506198190208</v>
       </c>
       <c r="AN19" t="n">
-        <v>0.5593504297680485</v>
+        <v>0.5593499924571995</v>
       </c>
       <c r="AO19" t="n">
-        <v>0.6778220534648677</v>
+        <v>0.6778222663532341</v>
       </c>
       <c r="AP19" t="n">
-        <v>0.7291841835590211</v>
+        <v>0.729184194156471</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0.6302518741819607</v>
+        <v>0.6302523310251144</v>
       </c>
       <c r="AR19" t="n">
-        <v>0.5124620435297096</v>
+        <v>0.5124621570844141</v>
       </c>
       <c r="AS19" t="n">
-        <v>0.602781669239001</v>
+        <v>0.6027803585490418</v>
       </c>
       <c r="AT19" t="n">
-        <v>1.046859935724021</v>
+        <v>1.046878278982171</v>
       </c>
     </row>
     <row r="20">
@@ -2824,139 +2824,139 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.061126127819699</v>
+        <v>1.061124689658579</v>
       </c>
       <c r="C20" t="n">
-        <v>1.062499717373288</v>
+        <v>1.062498157122811</v>
       </c>
       <c r="D20" t="n">
-        <v>1.195657988914142</v>
+        <v>1.195658282568019</v>
       </c>
       <c r="E20" t="n">
-        <v>1.184033854278919</v>
+        <v>1.184033595160696</v>
       </c>
       <c r="F20" t="n">
-        <v>1.382432107812416</v>
+        <v>1.382433727538489</v>
       </c>
       <c r="G20" t="n">
-        <v>1.137283957064241</v>
+        <v>1.137283592844397</v>
       </c>
       <c r="H20" t="n">
-        <v>1.162736083378001</v>
+        <v>1.162745376914049</v>
       </c>
       <c r="I20" t="n">
-        <v>1.253992355200363</v>
+        <v>1.253993976608952</v>
       </c>
       <c r="J20" t="n">
-        <v>1.182528064463374</v>
+        <v>1.182528637996505</v>
       </c>
       <c r="K20" t="n">
-        <v>0.8827579993057347</v>
+        <v>0.8827576748222491</v>
       </c>
       <c r="L20" t="n">
-        <v>0.9834326120483434</v>
+        <v>0.9834313361920108</v>
       </c>
       <c r="M20" t="n">
-        <v>1.128434641117982</v>
+        <v>1.12844159550798</v>
       </c>
       <c r="N20" t="n">
-        <v>1.094453185513187</v>
+        <v>1.094451527516665</v>
       </c>
       <c r="O20" t="n">
-        <v>1.207738805470905</v>
+        <v>1.207739345295294</v>
       </c>
       <c r="P20" t="n">
-        <v>0.8097695973210766</v>
+        <v>0.8097684987872942</v>
       </c>
       <c r="Q20" t="n">
-        <v>1.181679047957968</v>
+        <v>1.181677316589085</v>
       </c>
       <c r="R20" t="n">
-        <v>1.102471945413748</v>
+        <v>1.102469605943154</v>
       </c>
       <c r="S20" t="n">
-        <v>1.017738675050747</v>
+        <v>1.017746331075258</v>
       </c>
       <c r="T20" t="n">
-        <v>1.143651983992637</v>
+        <v>1.143654747725147</v>
       </c>
       <c r="U20" t="n">
-        <v>0.7150884391947429</v>
+        <v>0.7150872453490216</v>
       </c>
       <c r="V20" t="n">
-        <v>1.037165220828365</v>
+        <v>1.037166661325137</v>
       </c>
       <c r="W20" t="n">
-        <v>1.127372810265938</v>
+        <v>1.127373053423524</v>
       </c>
       <c r="X20" t="n">
-        <v>1.256144556143501</v>
+        <v>1.256144268187815</v>
       </c>
       <c r="Y20" t="n">
-        <v>1.229325022963012</v>
+        <v>1.229328906500203</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.267398787553067</v>
+        <v>1.26739866220571</v>
       </c>
       <c r="AA20" t="n">
-        <v>1.496879014251993</v>
+        <v>1.496879019408888</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.295561650833039</v>
+        <v>1.295562467749166</v>
       </c>
       <c r="AC20" t="n">
-        <v>1.088848158316566</v>
+        <v>1.088835768456003</v>
       </c>
       <c r="AD20" t="n">
-        <v>1.186182610163209</v>
+        <v>1.186182852980646</v>
       </c>
       <c r="AE20" t="n">
-        <v>1.304469486926644</v>
+        <v>1.304472267420899</v>
       </c>
       <c r="AF20" t="n">
-        <v>1.445819034921584</v>
+        <v>1.445816893476502</v>
       </c>
       <c r="AG20" t="n">
-        <v>1.394244946758477</v>
+        <v>1.394244833373323</v>
       </c>
       <c r="AH20" t="n">
-        <v>1.361086671583773</v>
+        <v>1.361085243062184</v>
       </c>
       <c r="AI20" t="n">
-        <v>0.9664455767685438</v>
+        <v>0.9664454875089763</v>
       </c>
       <c r="AJ20" t="n">
-        <v>1.479246144571493</v>
+        <v>1.4792458684209</v>
       </c>
       <c r="AK20" t="n">
-        <v>1.432204906843434</v>
+        <v>1.432204778160243</v>
       </c>
       <c r="AL20" t="n">
-        <v>1.09130928567161</v>
+        <v>1.091309325125577</v>
       </c>
       <c r="AM20" t="n">
-        <v>1.452041187613623</v>
+        <v>1.452041158386802</v>
       </c>
       <c r="AN20" t="n">
-        <v>1.440953792630096</v>
+        <v>1.440953355319248</v>
       </c>
       <c r="AO20" t="n">
-        <v>1.561819876002694</v>
+        <v>1.561820088891061</v>
       </c>
       <c r="AP20" t="n">
-        <v>1.665576625301137</v>
+        <v>1.665576635898587</v>
       </c>
       <c r="AQ20" t="n">
-        <v>1.520760325235596</v>
+        <v>1.52076078207875</v>
       </c>
       <c r="AR20" t="n">
-        <v>1.331601073088451</v>
+        <v>1.331601186643156</v>
       </c>
       <c r="AS20" t="n">
-        <v>1.45504026863953</v>
+        <v>1.45503895794957</v>
       </c>
       <c r="AT20" t="n">
-        <v>2.046859935724021</v>
+        <v>2.046878278982171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>